<commit_message>
Atualizacao das comissoes - 08/10/2026 08:35
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -814,28 +814,88 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="12">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
+      <c r="A11" s="7" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Leonardo de Carvalho Cruz</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Instalação do purificador</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0902</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="8" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
+      <c r="A12" s="7" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Leonardo de Carvalho Cruz</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Refil E3</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0902</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="12">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
+      <c r="A13" s="7" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Eliene</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Instalação do purificador</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0903</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="12">
       <c r="A14" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 08/10/2026 16:40
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -898,28 +898,88 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="12">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
+      <c r="A14" s="7" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Guiomar Macedo Freire - Antonio vila</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0041</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="12">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
+      <c r="A15" s="7" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Geisa Cunha Novais - Marcos</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Refil + Mangueira</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0270</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="12">
-      <c r="A16" s="7" t="n"/>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
+      <c r="A16" s="7" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Chapada Brindes</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Instalação do purificador</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>OUT-0102</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="12">
       <c r="A17" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 09/10/2026 11:57
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -982,28 +982,88 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="12">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
+      <c r="A17" s="7" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Rafael Landin Ribeiro</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0530</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="12">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
+      <c r="A18" s="7" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Restaurante Bonzão Bode - Aloisio Queiroz</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Refil Pro Life + Refil Universal</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento (metade paga no débito)</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0258</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="12">
-      <c r="A19" s="7" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
+      <c r="A19" s="7" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Tropical Motos LTDA</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Refil Pro Life</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0296</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="12">
       <c r="A20" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 10/10/2026 09:35
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1066,11 +1066,27 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="12">
-      <c r="A20" s="7" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
+      <c r="A20" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Josélia Nascimento da Silva Gomes</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
       <c r="F20" s="2" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="12">

</xml_diff>

<commit_message>
Atualizacao das comissoes - 10/10/2026 12:37
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1087,31 +1087,95 @@
           <t>Cartão</t>
         </is>
       </c>
-      <c r="F20" s="2" t="n"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0313</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="12">
-      <c r="A21" s="7" t="n"/>
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
+      <c r="A21" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Gabriela Araujo</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Instalação do purificador</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0038</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="12">
-      <c r="A22" s="7" t="n"/>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
+      <c r="A22" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Michelle Santos de Almeida Rocha</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Instalação do purificador</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0904</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="12">
-      <c r="A23" s="7" t="n"/>
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
+      <c r="A23" s="7" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Michelle Santos de Almeida Rocha</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Venda do Pré-filtro</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0904</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="12">
       <c r="A24" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 13/10/2026 14:48
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1178,20 +1178,60 @@
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="12">
-      <c r="A24" s="7" t="n"/>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
+      <c r="A24" s="7" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Leonardo Silva de Brito</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Refil + Mangueira + Limpeza do purificador</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>OUT-0103</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="12">
-      <c r="A25" s="7" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
+      <c r="A25" s="7" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Lorena Coelho</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Refil + Pré-filtro</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0905</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="12">
       <c r="A26" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 14/10/2026 11:58
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1234,11 +1234,27 @@
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="12">
-      <c r="A26" s="7" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
+      <c r="A26" s="7" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Olegario Oliveira da Silva</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Refil + Troca de peça (mangueira)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F26" s="2" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="12">

</xml_diff>

<commit_message>
Atualizacao das comissoes - 14/10/2026 17:41
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1258,36 +1258,116 @@
       <c r="F26" s="2" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="12">
-      <c r="A27" s="7" t="n"/>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="8" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
+      <c r="A27" s="7" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Aldaci Freire de Araujo</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0529</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="12">
-      <c r="A28" s="7" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
+      <c r="A28" s="7" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Marilia Silva</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0590</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="12">
-      <c r="A29" s="7" t="n"/>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
+      <c r="A29" s="7" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Marilia Silva</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Troca de peça (termostato)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0590</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="12">
-      <c r="A30" s="7" t="n"/>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="8" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
+      <c r="A30" s="7" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Reginaldo Novaes de Oliveira - Barbara Novais</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0524</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="12">
       <c r="A31" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 15/10/2026 11:27
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1370,20 +1370,60 @@
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="12">
-      <c r="A31" s="7" t="n"/>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="8" t="n"/>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
+      <c r="A31" s="7" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Casa das Portas Comercio de Madeiras LTDA</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0046</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="12">
-      <c r="A32" s="7" t="n"/>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="8" t="n"/>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
+      <c r="A32" s="7" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Casa do Construtor</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0320</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="12">
       <c r="A33" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 15/10/2026 18:22
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1426,20 +1426,60 @@
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="12">
-      <c r="A33" s="7" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="8" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
+      <c r="A33" s="7" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Edinaldo Nunes - Marilene de Souza Oliveira</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0499</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="12">
-      <c r="A34" s="7" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="8" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
+      <c r="A34" s="7" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Primeiro Tabelionato de Notas - Tatiana Miranda Siqueira</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0253</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="12">
       <c r="A35" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 16/10/2026 12:26
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1482,107 +1482,316 @@
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="12">
-      <c r="A35" s="7" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="8" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
+      <c r="A35" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Ages Educação Ltda</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
       <c r="F35" s="2" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="12">
-      <c r="A36" s="7" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="8" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
+      <c r="A36" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Ages Educação Ltda</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
       <c r="F36" s="2" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1" s="12">
-      <c r="A37" s="7" t="n"/>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="8" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
+      <c r="A37" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Ages Educação Ltda</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
       <c r="F37" s="2" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="12">
-      <c r="A38" s="7" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="8" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
+      <c r="A38" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Ages Educação Ltda</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
       <c r="F38" s="2" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="12">
-      <c r="A39" s="7" t="n"/>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="8" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="n"/>
+      <c r="A39" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Ages Educação Ltda</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
       <c r="F39" s="2" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="12">
-      <c r="A40" s="7" t="n"/>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="8" t="n"/>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="n"/>
+      <c r="A40" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
       <c r="F40" s="2" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="12">
-      <c r="A41" s="7" t="n"/>
-      <c r="B41" s="2" t="n"/>
-      <c r="C41" s="8" t="n"/>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="n"/>
+      <c r="A41" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
       <c r="F41" s="2" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="12">
-      <c r="A42" s="7" t="n"/>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="8" t="n"/>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="n"/>
+      <c r="A42" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
       <c r="F42" s="2" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="12">
-      <c r="A43" s="7" t="n"/>
-      <c r="B43" s="2" t="n"/>
-      <c r="C43" s="8" t="n"/>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="2" t="n"/>
+      <c r="A43" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
       <c r="F43" s="2" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1" s="12">
-      <c r="A44" s="7" t="n"/>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="8" t="n"/>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="n"/>
+      <c r="A44" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
       <c r="F44" s="2" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="12">
-      <c r="A45" s="7" t="n"/>
-      <c r="B45" s="2" t="n"/>
-      <c r="C45" s="8" t="n"/>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="n"/>
+      <c r="A45" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
       <c r="F45" s="2" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1" s="12">
-      <c r="A46" s="7" t="n"/>
-      <c r="B46" s="2" t="n"/>
-      <c r="C46" s="8" t="n"/>
-      <c r="D46" s="2" t="n"/>
-      <c r="E46" s="2" t="n"/>
+      <c r="A46" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
       <c r="F46" s="2" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1" s="12">
-      <c r="A47" s="7" t="n"/>
-      <c r="B47" s="2" t="n"/>
-      <c r="C47" s="8" t="n"/>
-      <c r="D47" s="2" t="n"/>
-      <c r="E47" s="2" t="n"/>
+      <c r="A47" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="12">
       <c r="A48" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 16/10/2026 17:59
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1444,7 +1444,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Dinheiro</t>
+          <t>Dinheiro + Pix</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Ages Educação Ltda</t>
+          <t>Ages Educação Ltda - Jacobina</t>
         </is>
       </c>
       <c r="C35" s="8" t="n">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Aguardando pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F35" s="2" t="n"/>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Ages Educação Ltda</t>
+          <t>Ages Educação Ltda - Jacobina</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Aguardando pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F36" s="2" t="n"/>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Ages Educação Ltda</t>
+          <t>Ages Educação Ltda - Jacobina</t>
         </is>
       </c>
       <c r="C37" s="8" t="n">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Aguardando pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F37" s="2" t="n"/>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Ages Educação Ltda</t>
+          <t>Ages Educação Ltda - Jacobina</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Aguardando pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F38" s="2" t="n"/>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Ages Educação Ltda</t>
+          <t>Ages Educação Ltda - Jacobina</t>
         </is>
       </c>
       <c r="C39" s="8" t="n">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Aguardando pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F39" s="2" t="n"/>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Aguardando pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F40" s="2" t="n"/>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Aguardando pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F41" s="2" t="n"/>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Aguardando pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F42" s="2" t="n"/>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Aguardando pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F43" s="2" t="n"/>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Aguardando pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F44" s="2" t="n"/>
@@ -1740,7 +1740,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Aguardando pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F45" s="2" t="n"/>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Aguardando pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F46" s="2" t="n"/>
@@ -1788,38 +1788,122 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="n"/>
+    </row>
+    <row r="48" ht="15" customHeight="1" s="12">
+      <c r="A48" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Alcina Rocha Lima Azevedo</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0033</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="15" customHeight="1" s="12">
+      <c r="A49" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>DFLL Serviços Medicos Ltda - ImCardio - Instituto Materno Cardiologico</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento (R$ 140 pago em dinheiro)</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0116</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15" customHeight="1" s="12">
+      <c r="A50" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Contabilidade Abreu</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Troca de peça (termostato)</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
           <t>Aguardando pagamento</t>
         </is>
       </c>
-      <c r="F47" s="2" t="n"/>
-    </row>
-    <row r="48" ht="15" customHeight="1" s="12">
-      <c r="A48" s="7" t="n"/>
-      <c r="B48" s="2" t="n"/>
-      <c r="C48" s="8" t="n"/>
-      <c r="D48" s="2" t="n"/>
-      <c r="E48" s="2" t="n"/>
-    </row>
-    <row r="49" ht="15" customHeight="1" s="12">
-      <c r="A49" s="7" t="n"/>
-      <c r="B49" s="2" t="n"/>
-      <c r="C49" s="8" t="n"/>
-      <c r="D49" s="2" t="n"/>
-      <c r="E49" s="2" t="n"/>
-    </row>
-    <row r="50" ht="15" customHeight="1" s="12">
-      <c r="A50" s="7" t="n"/>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="8" t="n"/>
-      <c r="D50" s="2" t="n"/>
-      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0105</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="12">
-      <c r="A51" s="7" t="n"/>
-      <c r="B51" s="2" t="n"/>
-      <c r="C51" s="8" t="n"/>
-      <c r="D51" s="2" t="n"/>
-      <c r="E51" s="2" t="n"/>
+      <c r="A51" s="7" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Eduardo Santos da Silva</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0408</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="12">
       <c r="A52" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 19/10/2026 09:17
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -691,1219 +691,391 @@
     </row>
     <row r="6" ht="15" customHeight="1" s="12">
       <c r="A6" s="7" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Carneiro Ultra Drogaria LTDA - Filial 01</t>
+          <t>Michelle Santos de Almeida Rocha</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Refil</t>
+          <t>Venda de pré-filtro — ficou da quinzena de 05/10 a 16/10 (pagar junto com a próxima)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Dinheiro</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n"/>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0904</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="12">
-      <c r="A7" s="7" t="n">
-        <v>46300</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Carneiro Ultra Drogaria LTDA - Filial 01</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Troca de peça (botões)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Dinheiro</t>
-        </is>
-      </c>
+      <c r="A7" s="7" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="12">
-      <c r="A8" s="7" t="n">
-        <v>46300</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Luiza Exdra Carneiro</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Cartão</t>
-        </is>
-      </c>
+      <c r="A8" s="7" t="n"/>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="12">
-      <c r="A9" s="7" t="n">
-        <v>46300</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Igreja Messianica Mundial do Brasil</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Aguardando pagamento</t>
-        </is>
-      </c>
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="12">
-      <c r="A10" s="7" t="n">
-        <v>46301</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Fiolaser Spa (Spa Requião Marques Ltda)</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Troca de peça (mangueira e conexão)</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Dinheiro</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>EMP-0319</t>
-        </is>
-      </c>
+      <c r="A10" s="7" t="n"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="12">
-      <c r="A11" s="7" t="n">
-        <v>46302</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Leonardo de Carvalho Cruz</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Instalação</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0902</t>
-        </is>
-      </c>
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="12">
-      <c r="A12" s="7" t="n">
-        <v>46302</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Leonardo de Carvalho Cruz</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0902</t>
-        </is>
-      </c>
+      <c r="A12" s="7" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="12">
-      <c r="A13" s="7" t="n">
-        <v>46302</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Eliene</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Instalação</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Cartão</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0903</t>
-        </is>
-      </c>
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="12">
-      <c r="A14" s="7" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Guiomar Macedo Freire - Antonio vila</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Cartão</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0041</t>
-        </is>
-      </c>
+      <c r="A14" s="7" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="12">
-      <c r="A15" s="7" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Geisa Cunha Novais - Marcos</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Refil + Troca de peça (mangueira)</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0270</t>
-        </is>
-      </c>
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="12">
-      <c r="A16" s="7" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Chapada Brindes</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Instalação</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>OUT-0102</t>
-        </is>
-      </c>
+      <c r="A16" s="7" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="12">
-      <c r="A17" s="7" t="n">
-        <v>46304</v>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Rafael Landin Ribeiro</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0530</t>
-        </is>
-      </c>
+      <c r="A17" s="7" t="n"/>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="12">
-      <c r="A18" s="7" t="n">
-        <v>46304</v>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Restaurante Bonzão Bode - Aloisio Queiroz</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Aguardando pagamento (metade paga no débito)</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>EMP-0258</t>
-        </is>
-      </c>
+      <c r="A18" s="7" t="n"/>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="12">
-      <c r="A19" s="7" t="n">
-        <v>46304</v>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Tropical Motos LTDA</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Aguardando pagamento</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>EMP-0296</t>
-        </is>
-      </c>
+      <c r="A19" s="7" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="12">
-      <c r="A20" s="7" t="n">
-        <v>46305</v>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Josélia Nascimento da Silva Gomes</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Cartão</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0313</t>
-        </is>
-      </c>
+      <c r="A20" s="7" t="n"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="12">
-      <c r="A21" s="7" t="n">
-        <v>46305</v>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Gabriela Araujo</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Instalação</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Cartão</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0038</t>
-        </is>
-      </c>
+      <c r="A21" s="7" t="n"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="12">
-      <c r="A22" s="7" t="n">
-        <v>46305</v>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Michelle Santos de Almeida Rocha</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Instalação</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Cartão</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0904</t>
-        </is>
-      </c>
+      <c r="A22" s="7" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="12">
-      <c r="A23" s="7" t="n">
-        <v>46305</v>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Michelle Santos de Almeida Rocha</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Venda de pré-filtro</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0904</t>
-        </is>
-      </c>
+      <c r="A23" s="7" t="n"/>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="12">
-      <c r="A24" s="7" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Leonardo Silva de Brito</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Refil + Troca de peça (mangueira) + Limpeza</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>OUT-0103</t>
-        </is>
-      </c>
+      <c r="A24" s="7" t="n"/>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="12">
-      <c r="A25" s="7" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Lorena Coelho</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Cartão</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0905</t>
-        </is>
-      </c>
+      <c r="A25" s="7" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="12">
-      <c r="A26" s="7" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Olegario Oliveira da Silva</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Refil + Troca de peça (mangueira)</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Dinheiro</t>
-        </is>
-      </c>
+      <c r="A26" s="7" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="12">
-      <c r="A27" s="7" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Aldaci Freire de Araujo</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>Dinheiro</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0529</t>
-        </is>
-      </c>
+      <c r="A27" s="7" t="n"/>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="12">
-      <c r="A28" s="7" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Marilia Silva</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Cartão</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0590</t>
-        </is>
-      </c>
+      <c r="A28" s="7" t="n"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="12">
-      <c r="A29" s="7" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Marilia Silva</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>Troca de peça (termostato)</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>Cartão</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0590</t>
-        </is>
-      </c>
+      <c r="A29" s="7" t="n"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="12">
-      <c r="A30" s="7" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Reginaldo Novaes de Oliveira - Barbara Novais</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Cartão</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0524</t>
-        </is>
-      </c>
+      <c r="A30" s="7" t="n"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="12">
-      <c r="A31" s="7" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Casa das Portas Comercio de Madeiras LTDA</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Dinheiro</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>EMP-0046</t>
-        </is>
-      </c>
+      <c r="A31" s="7" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1" s="12">
-      <c r="A32" s="7" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Casa do Construtor</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Aguardando pagamento</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>EMP-0320</t>
-        </is>
-      </c>
+      <c r="A32" s="7" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1" s="12">
-      <c r="A33" s="7" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Edinaldo Nunes - Marilene de Souza Oliveira</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Dinheiro + Pix</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0499</t>
-        </is>
-      </c>
+      <c r="A33" s="7" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="12">
-      <c r="A34" s="7" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Primeiro Tabelionato de Notas - Tatiana Miranda Siqueira</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>EMP-0253</t>
-        </is>
-      </c>
+      <c r="A34" s="7" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="8" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="12">
-      <c r="A35" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Ages Educação Ltda - Jacobina</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>Refil + pré-filtro (bebedouro IBBL)</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
+      <c r="A35" s="7" t="n"/>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="12">
-      <c r="A36" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Ages Educação Ltda - Jacobina</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>Refil + pré-filtro (bebedouro IBBL)</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
+      <c r="A36" s="7" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1" s="12">
-      <c r="A37" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Ages Educação Ltda - Jacobina</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>Refil + pré-filtro (bebedouro IBBL)</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
+      <c r="A37" s="7" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="12">
-      <c r="A38" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Ages Educação Ltda - Jacobina</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>Refil + pré-filtro (bebedouro IBBL)</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
+      <c r="A38" s="7" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="8" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="12">
-      <c r="A39" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Ages Educação Ltda - Jacobina</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
+      <c r="A39" s="7" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="8" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="12">
-      <c r="A40" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>CIS Jacobina</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>Refil + pré-filtro (bebedouro IBBL)</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
+      <c r="A40" s="7" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="8" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="12">
-      <c r="A41" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>CIS Jacobina</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>Refil + pré-filtro (bebedouro IBBL)</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
+      <c r="A41" s="7" t="n"/>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="8" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="12">
-      <c r="A42" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>CIS Jacobina</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Refil + pré-filtro (bebedouro IBBL)</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
+      <c r="A42" s="7" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="12">
-      <c r="A43" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>CIS Jacobina</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Refil + pré-filtro (bebedouro IBBL)</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
+      <c r="A43" s="7" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="8" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
       <c r="F43" s="2" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1" s="12">
-      <c r="A44" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>CIS Jacobina</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Refil + pré-filtro (bebedouro IBBL)</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
+      <c r="A44" s="7" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="8" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="12">
-      <c r="A45" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>CIS Jacobina</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>Refil + pré-filtro (bebedouro IBBL)</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
+      <c r="A45" s="7" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="8" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
       <c r="F45" s="2" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1" s="12">
-      <c r="A46" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>CIS Jacobina</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Refil + pré-filtro (bebedouro IBBL)</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
+      <c r="A46" s="7" t="n"/>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="8" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1" s="12">
-      <c r="A47" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>CIS Jacobina</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>Refil + pré-filtro (bebedouro IBBL)</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
+      <c r="A47" s="7" t="n"/>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="8" t="n"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="12">
-      <c r="A48" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Alcina Rocha Lima Azevedo</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Cartão</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0033</t>
-        </is>
-      </c>
+      <c r="A48" s="7" t="n"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="8" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1" s="12">
-      <c r="A49" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>DFLL Serviços Medicos Ltda - ImCardio - Instituto Materno Cardiologico</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Refil + pré-filtro</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>Aguardando pagamento (R$ 140 pago em dinheiro)</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>EMP-0116</t>
-        </is>
-      </c>
+      <c r="A49" s="7" t="n"/>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="8" t="n"/>
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
     </row>
     <row r="50" ht="15" customHeight="1" s="12">
-      <c r="A50" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Contabilidade Abreu</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Troca de peça (termostato)</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>Aguardando pagamento</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>EMP-0105</t>
-        </is>
-      </c>
+      <c r="A50" s="7" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="8" t="n"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
     </row>
     <row r="51" ht="15" customHeight="1" s="12">
-      <c r="A51" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>Eduardo Santos da Silva</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>Refil</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>Pix</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>CLI-0408</t>
-        </is>
-      </c>
+      <c r="A51" s="7" t="n"/>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="8" t="n"/>
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
     </row>
     <row r="52" ht="15" customHeight="1" s="12">
       <c r="A52" s="7" t="n"/>
@@ -11071,229 +10243,1534 @@
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="17" t="n"/>
-      <c r="C254" s="18" t="n"/>
-      <c r="G254" s="17" t="n"/>
+      <c r="A254" s="17" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Carneiro Ultra Drogaria LTDA - Filial 01</t>
+        </is>
+      </c>
+      <c r="C254" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G254" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="255">
-      <c r="A255" s="17" t="n"/>
-      <c r="C255" s="18" t="n"/>
-      <c r="G255" s="17" t="n"/>
+      <c r="A255" s="17" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Carneiro Ultra Drogaria LTDA - Filial 01</t>
+        </is>
+      </c>
+      <c r="C255" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Troca de peça (botões)</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G255" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="256">
-      <c r="A256" s="17" t="n"/>
-      <c r="C256" s="18" t="n"/>
-      <c r="G256" s="17" t="n"/>
+      <c r="A256" s="17" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Luiza Exdra Carneiro</t>
+        </is>
+      </c>
+      <c r="C256" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G256" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="257">
-      <c r="A257" s="17" t="n"/>
-      <c r="C257" s="18" t="n"/>
-      <c r="G257" s="17" t="n"/>
+      <c r="A257" s="17" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Igreja Messianica Mundial do Brasil</t>
+        </is>
+      </c>
+      <c r="C257" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G257" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="258">
-      <c r="A258" s="17" t="n"/>
-      <c r="C258" s="18" t="n"/>
-      <c r="G258" s="17" t="n"/>
+      <c r="A258" s="17" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Fiolaser Spa (Spa Requião Marques Ltda)</t>
+        </is>
+      </c>
+      <c r="C258" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Troca de peça (mangueira e conexão)</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G258" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>EMP-0319</t>
+        </is>
+      </c>
     </row>
     <row r="259">
-      <c r="A259" s="17" t="n"/>
-      <c r="C259" s="18" t="n"/>
-      <c r="G259" s="17" t="n"/>
+      <c r="A259" s="17" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Leonardo de Carvalho Cruz</t>
+        </is>
+      </c>
+      <c r="C259" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Instalação</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G259" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>CLI-0902</t>
+        </is>
+      </c>
     </row>
     <row r="260">
-      <c r="A260" s="17" t="n"/>
-      <c r="C260" s="18" t="n"/>
-      <c r="G260" s="17" t="n"/>
+      <c r="A260" s="17" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Leonardo de Carvalho Cruz</t>
+        </is>
+      </c>
+      <c r="C260" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G260" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>CLI-0902</t>
+        </is>
+      </c>
     </row>
     <row r="261">
-      <c r="A261" s="17" t="n"/>
-      <c r="C261" s="18" t="n"/>
-      <c r="G261" s="17" t="n"/>
+      <c r="A261" s="17" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Eliene</t>
+        </is>
+      </c>
+      <c r="C261" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Instalação</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G261" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>CLI-0903</t>
+        </is>
+      </c>
     </row>
     <row r="262">
-      <c r="A262" s="17" t="n"/>
-      <c r="C262" s="18" t="n"/>
-      <c r="G262" s="17" t="n"/>
+      <c r="A262" s="17" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Guiomar Macedo Freire - Antonio vila</t>
+        </is>
+      </c>
+      <c r="C262" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G262" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>CLI-0041</t>
+        </is>
+      </c>
     </row>
     <row r="263">
-      <c r="A263" s="17" t="n"/>
-      <c r="C263" s="18" t="n"/>
-      <c r="G263" s="17" t="n"/>
+      <c r="A263" s="17" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Geisa Cunha Novais - Marcos</t>
+        </is>
+      </c>
+      <c r="C263" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Refil + Troca de peça (mangueira)</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G263" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>CLI-0270</t>
+        </is>
+      </c>
     </row>
     <row r="264">
-      <c r="A264" s="17" t="n"/>
-      <c r="C264" s="18" t="n"/>
-      <c r="G264" s="17" t="n"/>
+      <c r="A264" s="17" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Chapada Brindes</t>
+        </is>
+      </c>
+      <c r="C264" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Instalação</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G264" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>OUT-0102</t>
+        </is>
+      </c>
     </row>
     <row r="265">
-      <c r="A265" s="17" t="n"/>
-      <c r="C265" s="18" t="n"/>
-      <c r="G265" s="17" t="n"/>
+      <c r="A265" s="17" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Rafael Landin Ribeiro</t>
+        </is>
+      </c>
+      <c r="C265" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G265" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>CLI-0530</t>
+        </is>
+      </c>
     </row>
     <row r="266">
-      <c r="A266" s="17" t="n"/>
-      <c r="C266" s="18" t="n"/>
-      <c r="G266" s="17" t="n"/>
+      <c r="A266" s="17" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Restaurante Bonzão Bode - Aloisio Queiroz</t>
+        </is>
+      </c>
+      <c r="C266" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento (metade paga no débito)</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G266" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>EMP-0258</t>
+        </is>
+      </c>
     </row>
     <row r="267">
-      <c r="A267" s="17" t="n"/>
-      <c r="C267" s="18" t="n"/>
-      <c r="G267" s="17" t="n"/>
+      <c r="A267" s="17" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Tropical Motos LTDA</t>
+        </is>
+      </c>
+      <c r="C267" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G267" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>EMP-0296</t>
+        </is>
+      </c>
     </row>
     <row r="268">
-      <c r="A268" s="17" t="n"/>
-      <c r="C268" s="18" t="n"/>
-      <c r="G268" s="17" t="n"/>
+      <c r="A268" s="17" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Josélia Nascimento da Silva Gomes</t>
+        </is>
+      </c>
+      <c r="C268" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G268" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>CLI-0313</t>
+        </is>
+      </c>
     </row>
     <row r="269">
-      <c r="A269" s="17" t="n"/>
-      <c r="C269" s="18" t="n"/>
-      <c r="G269" s="17" t="n"/>
+      <c r="A269" s="17" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Gabriela Araujo</t>
+        </is>
+      </c>
+      <c r="C269" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Instalação</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G269" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>CLI-0038</t>
+        </is>
+      </c>
     </row>
     <row r="270">
-      <c r="A270" s="17" t="n"/>
-      <c r="C270" s="18" t="n"/>
-      <c r="G270" s="17" t="n"/>
+      <c r="A270" s="17" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Michelle Santos de Almeida Rocha</t>
+        </is>
+      </c>
+      <c r="C270" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Instalação</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G270" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>CLI-0904</t>
+        </is>
+      </c>
     </row>
     <row r="271">
-      <c r="A271" s="17" t="n"/>
-      <c r="C271" s="18" t="n"/>
-      <c r="G271" s="17" t="n"/>
+      <c r="A271" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Leonardo Silva de Brito</t>
+        </is>
+      </c>
+      <c r="C271" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Refil + Troca de peça (mangueira) + Limpeza</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G271" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>OUT-0103</t>
+        </is>
+      </c>
     </row>
     <row r="272">
-      <c r="A272" s="17" t="n"/>
-      <c r="C272" s="18" t="n"/>
-      <c r="G272" s="17" t="n"/>
+      <c r="A272" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Lorena Coelho</t>
+        </is>
+      </c>
+      <c r="C272" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G272" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>CLI-0905</t>
+        </is>
+      </c>
     </row>
     <row r="273">
-      <c r="A273" s="17" t="n"/>
-      <c r="C273" s="18" t="n"/>
-      <c r="G273" s="17" t="n"/>
+      <c r="A273" s="17" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Olegario Oliveira da Silva</t>
+        </is>
+      </c>
+      <c r="C273" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Refil + Troca de peça (mangueira)</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G273" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="274">
-      <c r="A274" s="17" t="n"/>
-      <c r="C274" s="18" t="n"/>
-      <c r="G274" s="17" t="n"/>
+      <c r="A274" s="17" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Aldaci Freire de Araujo</t>
+        </is>
+      </c>
+      <c r="C274" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G274" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>CLI-0529</t>
+        </is>
+      </c>
     </row>
     <row r="275">
-      <c r="A275" s="17" t="n"/>
-      <c r="C275" s="18" t="n"/>
-      <c r="G275" s="17" t="n"/>
+      <c r="A275" s="17" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Marilia Silva</t>
+        </is>
+      </c>
+      <c r="C275" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G275" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>CLI-0590</t>
+        </is>
+      </c>
     </row>
     <row r="276">
-      <c r="A276" s="17" t="n"/>
-      <c r="C276" s="18" t="n"/>
-      <c r="G276" s="17" t="n"/>
+      <c r="A276" s="17" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Marilia Silva</t>
+        </is>
+      </c>
+      <c r="C276" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Troca de peça (termostato)</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G276" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>CLI-0590</t>
+        </is>
+      </c>
     </row>
     <row r="277">
-      <c r="A277" s="17" t="n"/>
-      <c r="C277" s="18" t="n"/>
-      <c r="G277" s="17" t="n"/>
+      <c r="A277" s="17" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Reginaldo Novaes de Oliveira - Barbara Novais</t>
+        </is>
+      </c>
+      <c r="C277" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G277" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>CLI-0524</t>
+        </is>
+      </c>
     </row>
     <row r="278">
-      <c r="A278" s="17" t="n"/>
-      <c r="C278" s="18" t="n"/>
-      <c r="G278" s="17" t="n"/>
+      <c r="A278" s="17" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Casa das Portas Comercio de Madeiras LTDA</t>
+        </is>
+      </c>
+      <c r="C278" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G278" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>EMP-0046</t>
+        </is>
+      </c>
     </row>
     <row r="279">
-      <c r="A279" s="17" t="n"/>
-      <c r="C279" s="18" t="n"/>
-      <c r="G279" s="17" t="n"/>
+      <c r="A279" s="17" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Casa do Construtor</t>
+        </is>
+      </c>
+      <c r="C279" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G279" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>EMP-0320</t>
+        </is>
+      </c>
     </row>
     <row r="280">
-      <c r="A280" s="17" t="n"/>
-      <c r="C280" s="18" t="n"/>
-      <c r="G280" s="17" t="n"/>
+      <c r="A280" s="17" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Edinaldo Nunes - Marilene de Souza Oliveira</t>
+        </is>
+      </c>
+      <c r="C280" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Dinheiro + Pix</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G280" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>CLI-0499</t>
+        </is>
+      </c>
     </row>
     <row r="281">
-      <c r="A281" s="17" t="n"/>
-      <c r="C281" s="18" t="n"/>
-      <c r="G281" s="17" t="n"/>
+      <c r="A281" s="17" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Primeiro Tabelionato de Notas - Tatiana Miranda Siqueira</t>
+        </is>
+      </c>
+      <c r="C281" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G281" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>EMP-0253</t>
+        </is>
+      </c>
     </row>
     <row r="282">
-      <c r="A282" s="17" t="n"/>
-      <c r="C282" s="18" t="n"/>
-      <c r="G282" s="17" t="n"/>
+      <c r="A282" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Ages Educação Ltda - Jacobina</t>
+        </is>
+      </c>
+      <c r="C282" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G282" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="283">
-      <c r="A283" s="17" t="n"/>
-      <c r="C283" s="18" t="n"/>
-      <c r="G283" s="17" t="n"/>
+      <c r="A283" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Ages Educação Ltda - Jacobina</t>
+        </is>
+      </c>
+      <c r="C283" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G283" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="284">
-      <c r="A284" s="17" t="n"/>
-      <c r="C284" s="18" t="n"/>
-      <c r="G284" s="17" t="n"/>
+      <c r="A284" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Ages Educação Ltda - Jacobina</t>
+        </is>
+      </c>
+      <c r="C284" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G284" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="285">
-      <c r="A285" s="17" t="n"/>
-      <c r="C285" s="18" t="n"/>
-      <c r="G285" s="17" t="n"/>
+      <c r="A285" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Ages Educação Ltda - Jacobina</t>
+        </is>
+      </c>
+      <c r="C285" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G285" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="286">
-      <c r="A286" s="17" t="n"/>
-      <c r="C286" s="18" t="n"/>
-      <c r="G286" s="17" t="n"/>
+      <c r="A286" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Ages Educação Ltda - Jacobina</t>
+        </is>
+      </c>
+      <c r="C286" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G286" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="287">
-      <c r="A287" s="17" t="n"/>
-      <c r="C287" s="18" t="n"/>
-      <c r="G287" s="17" t="n"/>
+      <c r="A287" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C287" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G287" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="288">
-      <c r="A288" s="17" t="n"/>
-      <c r="C288" s="18" t="n"/>
-      <c r="G288" s="17" t="n"/>
+      <c r="A288" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C288" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G288" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="289">
-      <c r="A289" s="17" t="n"/>
-      <c r="C289" s="18" t="n"/>
-      <c r="G289" s="17" t="n"/>
+      <c r="A289" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C289" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G289" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="290">
-      <c r="A290" s="17" t="n"/>
-      <c r="C290" s="18" t="n"/>
-      <c r="G290" s="17" t="n"/>
+      <c r="A290" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C290" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G290" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="291">
-      <c r="A291" s="17" t="n"/>
-      <c r="C291" s="18" t="n"/>
-      <c r="G291" s="17" t="n"/>
+      <c r="A291" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C291" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G291" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="292">
-      <c r="A292" s="17" t="n"/>
-      <c r="C292" s="18" t="n"/>
-      <c r="G292" s="17" t="n"/>
+      <c r="A292" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C292" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G292" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="293">
-      <c r="A293" s="17" t="n"/>
-      <c r="C293" s="18" t="n"/>
-      <c r="G293" s="17" t="n"/>
+      <c r="A293" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C293" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G293" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="294">
-      <c r="A294" s="17" t="n"/>
-      <c r="C294" s="18" t="n"/>
-      <c r="G294" s="17" t="n"/>
+      <c r="A294" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>CIS Jacobina</t>
+        </is>
+      </c>
+      <c r="C294" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro (bebedouro IBBL)</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G294" s="17" t="n">
+        <v>46312</v>
+      </c>
     </row>
     <row r="295">
-      <c r="A295" s="17" t="n"/>
-      <c r="C295" s="18" t="n"/>
-      <c r="G295" s="17" t="n"/>
+      <c r="A295" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Alcina Rocha Lima Azevedo</t>
+        </is>
+      </c>
+      <c r="C295" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G295" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>CLI-0033</t>
+        </is>
+      </c>
     </row>
     <row r="296">
-      <c r="A296" s="17" t="n"/>
-      <c r="C296" s="18" t="n"/>
-      <c r="G296" s="17" t="n"/>
+      <c r="A296" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>DFLL Serviços Medicos Ltda - ImCardio - Instituto Materno Cardiologico</t>
+        </is>
+      </c>
+      <c r="C296" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Refil + pré-filtro</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento (R$ 140 pago em dinheiro)</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G296" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>EMP-0116</t>
+        </is>
+      </c>
     </row>
     <row r="297">
-      <c r="A297" s="17" t="n"/>
-      <c r="C297" s="18" t="n"/>
-      <c r="G297" s="17" t="n"/>
+      <c r="A297" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Contabilidade Abreu</t>
+        </is>
+      </c>
+      <c r="C297" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Troca de peça (termostato)</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G297" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>EMP-0105</t>
+        </is>
+      </c>
     </row>
     <row r="298">
-      <c r="A298" s="17" t="n"/>
-      <c r="C298" s="18" t="n"/>
-      <c r="G298" s="17" t="n"/>
+      <c r="A298" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Eduardo Santos da Silva</t>
+        </is>
+      </c>
+      <c r="C298" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G298" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>CLI-0408</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="17" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 19/10/2026 18:29
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -718,76 +718,256 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="12">
-      <c r="A7" s="7" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
+      <c r="A7" s="7" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Carneiro Ultra Drogaria LTDA - Filial 02</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0043</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="12">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="8" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
+      <c r="A8" s="7" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Otica Imagem - José Luciano Viera Costa</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0238</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="12">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
+      <c r="A9" s="7" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Otica Imagem - José Luciano Viera Costa 1 Andar</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0238</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="12">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="8" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
+      <c r="A10" s="7" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Pedras e Pisos - Loja</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0245</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="12">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
+      <c r="A11" s="7" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Marsilia Marmores e Granitos Erelli</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0216</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="8" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
+      <c r="A12" s="7" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>A. S. Supermercado</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0321</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="12">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
+      <c r="A13" s="7" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Gilberto de Aguiar</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0629</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="12">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
+      <c r="A14" s="7" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Raulino Gonçalves dos Santos</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Instalação</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0906</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="12">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
+      <c r="A15" s="7" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Larissa Sena</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0907</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="12">
       <c r="A16" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 20/10/2026 12:19
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -691,29 +691,29 @@
     </row>
     <row r="6" ht="15" customHeight="1" s="12">
       <c r="A6" s="7" t="n">
-        <v>46305</v>
+        <v>46314</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Michelle Santos de Almeida Rocha</t>
+          <t>Carneiro Ultra Drogaria LTDA - Filial 02</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Venda de pré-filtro — ficou da quinzena de 05/10 a 16/10 (pagar junto com a próxima)</t>
+          <t>Refil</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Pix</t>
+          <t>Dinheiro</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>CLI-0904</t>
+          <t>EMP-0043</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Carneiro Ultra Drogaria LTDA - Filial 02</t>
+          <t>Otica Imagem - José Luciano Viera Costa</t>
         </is>
       </c>
       <c r="C7" s="8" t="n">
@@ -741,7 +741,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>EMP-0043</t>
+          <t>EMP-0238</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Otica Imagem - José Luciano Viera Costa</t>
+          <t>Otica Imagem - José Luciano Viera Costa 1 Andar</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
@@ -779,7 +779,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Otica Imagem - José Luciano Viera Costa 1 Andar</t>
+          <t>Pedras e Pisos - Loja</t>
         </is>
       </c>
       <c r="C9" s="8" t="n">
@@ -797,7 +797,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>EMP-0238</t>
+          <t>EMP-0245</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Pedras e Pisos - Loja</t>
+          <t>Marsilia Marmores e Granitos Erelli</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
@@ -820,12 +820,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Dinheiro</t>
+          <t>Aguardando pagamento</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>EMP-0245</t>
+          <t>EMP-0216</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Marsilia Marmores e Granitos Erelli</t>
+          <t>A. S. Supermercado</t>
         </is>
       </c>
       <c r="C11" s="8" t="n">
@@ -848,12 +848,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Aguardando pagamento</t>
+          <t>Dinheiro</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>EMP-0216</t>
+          <t>EMP-0321</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>A. S. Supermercado</t>
+          <t>Gilberto de Aguiar</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
@@ -881,7 +881,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>EMP-0321</t>
+          <t>CLI-0629</t>
         </is>
       </c>
     </row>
@@ -891,25 +891,25 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Gilberto de Aguiar</t>
+          <t>Raulino Gonçalves dos Santos</t>
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Refil</t>
+          <t>Instalação</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Dinheiro</t>
+          <t>Cartão</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>CLI-0629</t>
+          <t>CLI-0906</t>
         </is>
       </c>
     </row>
@@ -919,35 +919,35 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Raulino Gonçalves dos Santos</t>
+          <t>Larissa Sena</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Instalação</t>
+          <t>Refil</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Cartão</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>CLI-0906</t>
+          <t>CLI-0907</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="12">
       <c r="A15" s="7" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Larissa Sena</t>
+          <t>Int Odontologia - Larissa Sena</t>
         </is>
       </c>
       <c r="C15" s="8" t="n">
@@ -965,17 +965,37 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>CLI-0907</t>
+          <t>EMP-0184</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="12">
-      <c r="A16" s="7" t="n"/>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
+      <c r="A16" s="7" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Banco do Nordeste do Brasil</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0220</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="12">
       <c r="A17" s="7" t="n"/>
@@ -11953,9 +11973,40 @@
       </c>
     </row>
     <row r="299">
-      <c r="A299" s="17" t="n"/>
-      <c r="C299" s="18" t="n"/>
-      <c r="G299" s="17" t="n"/>
+      <c r="A299" s="17" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Michelle Santos de Almeida Rocha</t>
+        </is>
+      </c>
+      <c r="C299" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Venda de pré-filtro</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Quinzena de 05/10 a 16/10/2026</t>
+        </is>
+      </c>
+      <c r="G299" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>CLI-0904</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="17" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 20/10/2026 18:22
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -998,43 +998,139 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="12">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
+      <c r="A17" s="7" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Magna dos Santos Carneiro Goncalves - Mirna</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0488</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="12">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
+      <c r="A18" s="7" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Real Calçados Loja 1</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0255</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="12">
-      <c r="A19" s="7" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
+      <c r="A19" s="7" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Real Calçados Loja 1</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0255</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="12">
-      <c r="A20" s="7" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
+      <c r="A20" s="7" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Real Calçados Loja 1</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0255</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="12">
-      <c r="A21" s="7" t="n"/>
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
+      <c r="A21" s="7" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Loja da Claro</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
       <c r="F21" s="2" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="12">

</xml_diff>

<commit_message>
Atualizacao das comissoes - 21/10/2026 12:08
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1134,20 +1134,60 @@
       <c r="F21" s="2" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="12">
-      <c r="A22" s="7" t="n"/>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
+      <c r="A22" s="7" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Eliane Lisboa Silva</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0908</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="12">
-      <c r="A23" s="7" t="n"/>
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
+      <c r="A23" s="7" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Studio Malena Lorrane</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0283</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="12">
       <c r="A24" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 21/10/2026 14:35
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1190,12 +1190,32 @@
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="12">
-      <c r="A24" s="7" t="n"/>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
+      <c r="A24" s="7" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Miralva Lopes da Silva</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0390</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="12">
       <c r="A25" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 22/10/2026 18:17
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -12098,7 +12098,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Eduardo Santos da Silva</t>
+          <t>Tania Dourado - Eduardo Dourado</t>
         </is>
       </c>
       <c r="C298" s="18" t="n">
@@ -12124,7 +12124,7 @@
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>CLI-0408</t>
+          <t>CLI-0525</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 23/10/2026 12:03
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1218,19 +1218,51 @@
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="12">
-      <c r="A25" s="7" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
+      <c r="A25" s="7" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Alessandra Carvalho Vieira - Paulo Sergio</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F25" s="2" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="12">
-      <c r="A26" s="7" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
+      <c r="A26" s="7" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Rita Mesquita</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
       <c r="F26" s="2" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="12">

</xml_diff>

<commit_message>
Atualizacao das comissoes - 24/10/2026 10:19
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1266,11 +1266,27 @@
       <c r="F26" s="2" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="12">
-      <c r="A27" s="7" t="n"/>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="8" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
+      <c r="A27" s="7" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Leda Goretti Andrade Alves</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Limpeza</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
       <c r="F27" s="2" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="12">

</xml_diff>

<commit_message>
Atualizacao das comissoes - 26/10/2026 12:12
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1290,36 +1290,116 @@
       <c r="F27" s="2" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="12">
-      <c r="A28" s="7" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
+      <c r="A28" s="7" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Zelia Bernadete de Jesus</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0427</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="12">
-      <c r="A29" s="7" t="n"/>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
+      <c r="A29" s="7" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Patricio Rodrigues de Melo</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0440</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="12">
-      <c r="A30" s="7" t="n"/>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="8" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
+      <c r="A30" s="7" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Erlene Mendes</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0500</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="12">
-      <c r="A31" s="7" t="n"/>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="8" t="n"/>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
+      <c r="A31" s="7" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Fernanda Barreto - Marjore Barreto</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Cartão</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0221</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="12">
       <c r="A32" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 27/10/2026 12:14
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1402,12 +1402,32 @@
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="12">
-      <c r="A32" s="7" t="n"/>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="8" t="n"/>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
+      <c r="A32" s="7" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Vivencie Turismo Agencia de Viagens - Aneildes Rios</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Instalação de regulador de pressão</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0032</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="12">
       <c r="A33" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 27/10/2026 17:46
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1430,12 +1430,32 @@
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="12">
-      <c r="A33" s="7" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="8" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
+      <c r="A33" s="7" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Adriana Carvalho Sampaio - Jacobina Automoveis</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Instalação</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0479</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="12">
       <c r="A34" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 28/10/2026 17:28
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1458,28 +1458,88 @@
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="12">
-      <c r="A34" s="7" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="8" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
+      <c r="A34" s="7" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Clinica Amo - Mesquita Maia Atendimento Medico</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Troca de botões do purificador</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0068</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="12">
-      <c r="A35" s="7" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="8" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
+      <c r="A35" s="7" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Marineuza Goveia da Silva</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Pix + Dinheiro</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0497</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="12">
-      <c r="A36" s="7" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="8" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
+      <c r="A36" s="7" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Nara Goveia da Silva</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0496</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="12">
       <c r="A37" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 30/10/2026 12:10
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1542,28 +1542,88 @@
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="12">
-      <c r="A37" s="7" t="n"/>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="8" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
+      <c r="A37" s="7" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Kiely Midori Nascimento kataoka</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0551</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="12">
-      <c r="A38" s="7" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="8" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
+      <c r="A38" s="7" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Denise Vasconcelos Fernandes - Trat Fisio</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0114</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="12">
-      <c r="A39" s="7" t="n"/>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="8" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="n"/>
+      <c r="A39" s="7" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Central Mix Variedades EIRELI</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>EMP-0056</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="12">
       <c r="A40" s="7" t="n"/>

</xml_diff>

<commit_message>
Atualizacao das comissoes - 30/10/2026 17:06
</commit_message>
<xml_diff>
--- a/2026.xlsx
+++ b/2026.xlsx
@@ -1626,20 +1626,60 @@
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="12">
-      <c r="A40" s="7" t="n"/>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="8" t="n"/>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="2" t="n"/>
+      <c r="A40" s="7" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>João José da Silva Santos - Benedita da Silva</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0489</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="12">
-      <c r="A41" s="7" t="n"/>
-      <c r="B41" s="2" t="n"/>
-      <c r="C41" s="8" t="n"/>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="n"/>
+      <c r="A41" s="7" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Antonieta Alves da Silva</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Refil</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando pagamento</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>CLI-0540</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="12">
       <c r="A42" s="7" t="n"/>

</xml_diff>